<commit_message>
Updated as per api and docker image
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -455,7 +455,7 @@
         <v>615</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2252275</v>
+        <v>0.00615</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         <v>17346</v>
       </c>
       <c r="C3" t="n">
-        <v>0.70675</v>
+        <v>0.11846</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         <v>1300</v>
       </c>
       <c r="C4" t="n">
-        <v>0.66595</v>
+        <v>0.007000000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         <v>93</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2207905</v>
+        <v>0.0009299999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         <v>1079</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5591715</v>
+        <v>0.01079</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         <v>15631</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7152500000000001</v>
+        <v>0.09119000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         <v>148</v>
       </c>
       <c r="C8" t="n">
-        <v>0.551258</v>
+        <v>0.00148</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         <v>20000</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7200000000000001</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +559,7 @@
         <v>8000</v>
       </c>
       <c r="C10" t="n">
-        <v>0.6180000000000001</v>
+        <v>0.08000000000000002</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         <v>8500</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7322500000000001</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated demand fulfilment & capacity utilization logic, set default params after meet
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,131 +448,1236 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1225221615008QXC10</t>
+          <t>1225119015010QSTL0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>615</v>
+        <v>1703</v>
       </c>
       <c r="C2" t="n">
-        <v>0.00615</v>
+        <v>0.006192727272727273</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1225221715115SSTL0</t>
+          <t>1225121715115SSTL0</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17346</v>
+        <v>5668</v>
       </c>
       <c r="C3" t="n">
-        <v>0.11846</v>
+        <v>0.02061090909090909</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1225221716010SXC10</t>
+          <t>1225121716010SXC10</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1300</v>
+        <v>1941</v>
       </c>
       <c r="C4" t="n">
-        <v>0.007000000000000001</v>
+        <v>0.5014545454545455</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1225222615008RXC10</t>
+          <t>1225121Z14112LSTL0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>93</v>
+        <v>1802</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0009299999999999999</v>
+        <v>0.006552727272727273</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1225222716121MXC11</t>
+          <t>1225170015010LSTL0</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1079</v>
+        <v>6500</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01079</v>
+        <v>0.5236363636363637</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1225223516121PSKP0</t>
+          <t>1225170015012LSTL0</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15631</v>
+        <v>58111</v>
       </c>
       <c r="C7" t="n">
-        <v>0.09119000000000001</v>
+        <v>0.5636363636363636</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1325114613071TTMX0</t>
+          <t>1225175016012NJTL0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="C8" t="n">
-        <v>0.00148</v>
+        <v>0.417259393939394</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1325114812074TUHL0</t>
+          <t>1225219015008SLTB0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20000</v>
+        <v>300</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2</v>
+        <v>0.4177575757575758</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1325119015008SRBT0</t>
+          <t>1225219015010QSTL0</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8000</v>
+        <v>2900</v>
       </c>
       <c r="C10" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.01054545454545455</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>1225220Z16008RXC10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.416739393939394</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1225221615008QXC10</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>615</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4189030303030303</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1225221715115SSTL0</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>17346</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1225221716010SXC10</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5025454545454545</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1225222615008RXC10</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>93</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.4170048484848485</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1225222716121MXC11</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1079</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.003923636363636364</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1225223516121PSKP0</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>15631</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.5236363636363637</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1325114613071TTMX0</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>148</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.0005381818181818182</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1325114812074TUHL0</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.07272727272727274</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1325119015008SRBT0</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.02909090909090909</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>1325119815106QBRQ0</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>8500</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.08500000000000001</v>
+      <c r="B21" t="n">
+        <v>8533</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5309090909090909</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1325121715100SBRT0</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.02181818181818182</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1325121715100SRBT0</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.01818181818181818</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1325121715100SRXT0</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.01818181818181818</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1325121715115SLTB0</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.01818181818181818</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1325123715105SBRT0</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.02909090909090909</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1325123715105SRXT0</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>900</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.003272727272727273</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1325213612065SULX1</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2190</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1325213615099MSXT0</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>6300</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.5229090909090909</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1325214613071TTMX0</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2914</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.01059636363636364</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1325214812074TUHL0</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1325214813075STMX0</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3887</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.01413454545454546</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1325214813075SUNE1</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1325215513073TUHL0</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6055</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.02201818181818182</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1325215613075TTMX0</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.01818181818181818</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1325215613075TUHL0</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>9200</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.03345454545454545</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1325215813079STMX0</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>15030</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.4167757575757576</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1325215813079SUHL0</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.04363636363636364</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1325216513077TUHL0</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3005</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.01092727272727273</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1325216514079TTMX0</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5418</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.417030303030303</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1325216614081STMX0</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.06545454545454546</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1325216614081SUTR0</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5866</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.02133090909090909</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1325216814085STMX0</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.07272727272727274</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1325216814085SUTR0</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>5181</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.01884</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1325216814085TURL0</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>6853</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.4229939393939394</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1325216814085TURS0</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>300</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.001090909090909091</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1325217413077TUSP0</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.01818181818181818</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1325217415081HUTR0</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.01454545454545455</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1325217514082HURP0</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>421</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.001530909090909091</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1325217514082TTMX0</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>6562</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.4169212121212121</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1325217514082TUTR0</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.01818181818181818</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1325217514082TVECH</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2253</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.5029854545454545</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1325217515084HURP0</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>148</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.0005381818181818182</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1325217613082TUNE2</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>423</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.4182048484848485</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1325217614084HURL1</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1379</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.005014545454545456</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1325218415084TTMX0</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1557</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.005661818181818182</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1325218515088HTMX0</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>22300</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.4177575757575758</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1325218515088HURP0</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>456</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.001658181818181818</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1325218515088HUTR0</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4924</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.01790545454545455</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1325218515088TURL0</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2136</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.007767272727272727</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1325218515088TURS0</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>300</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0.001090909090909091</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1325218614088HURL0</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>3426</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0.4173939393939394</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1325219316087VURL0</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.02909090909090909</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1325219316087VURP0</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>609</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0.002214545454545455</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1325219316087VUTR0</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0.02545454545454545</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1325219416089HRHE0</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>17024</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0.5254545454545454</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1325220316091VURL1</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2004</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0.007287272727272727</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1325220416092VURL0</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>558</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0.002029090909090909</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1325220416092VURP0</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>11</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0.4167066666666667</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1325220515094VTMX0</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2261</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0.417030303030303</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1325220515094VURL1</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>93</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0.4170048484848485</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1325220515094VUTR0</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>6098</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0.02217454545454546</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1325220516095HTMX0</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2619</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0.4168484848484849</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1325220516095HUTR0</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0.02909090909090909</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1325221317098VUX10</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>4</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1.454545454545455e-05</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1325221416095VURL0</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>15005</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0.4166848484848485</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1325221416095VURS0</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>300</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0.001090909090909091</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1325221417100HURL1</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0.06545454545454546</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1325221417100HURS0</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>300</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0.001090909090909091</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1325221715100SRHT0</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0.07272727272727274</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1325221715100SRXT0</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0.01454545454545455</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1325222317101VUX10</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>172</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0.4172448484848485</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1325222417099HURL0</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2059</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0.4167757575757576</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1325223517104HRHT0</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>8030</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0.4167757575757576</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1325223517104HRPG0</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>579</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0.002105454545454545</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1325223616105HRHT0</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>2847</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0.01035272727272727</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1325223715105SRXT0</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>3256</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0.01184</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1325223916120QRAB0</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1160</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0.4208848484848485</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1325226517112HRHT0</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>3077</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0.419139393939394</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1425118916008QRBT0</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0.03272727272727273</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1D25115013008QXPC0</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>548</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0.001992727272727273</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1D25212812074FXC10</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>23400</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0.5850909090909091</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1D25212812086FXPC0</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>27500</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1D25213812090FXPC0</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>30700</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0.6116363636363636</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1D25214012006QXC10</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>500</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0.001818181818181818</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1D25215Z13008QXPC0</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>11264</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0.5181818181818182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Machine Utilization exclusions, CT (NA) value, complete machine schedule ouptut
</commit_message>
<xml_diff>
--- a/load_demand.xlsx
+++ b/load_demand.xlsx
@@ -443,7 +443,7 @@
         <v>1703</v>
       </c>
       <c r="C2" t="n">
-        <v>4.544187082821346e-05</v>
+        <v>0.004566908018235452</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,7 @@
         <v>5668</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0001512416464206188</v>
+        <v>0.01519978546527219</v>
       </c>
     </row>
     <row r="4">
@@ -469,7 +469,7 @@
         <v>1991</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9950368831626262</v>
+        <v>0.501206757843926</v>
       </c>
     </row>
     <row r="5">
@@ -482,7 +482,7 @@
         <v>1787</v>
       </c>
       <c r="C5" t="n">
-        <v>4.768327843218875e-05</v>
+        <v>0.004792169482434969</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
         <v>5200</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9951636294259462</v>
+        <v>0.5139447573075892</v>
       </c>
     </row>
     <row r="7">
@@ -508,7 +508,7 @@
         <v>65500</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9954384686916717</v>
+        <v>0.5415661035130062</v>
       </c>
     </row>
     <row r="8">
@@ -521,7 +521,7 @@
         <v>346</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8291966288162299</v>
+        <v>0.4175945293644409</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         <v>2900</v>
       </c>
       <c r="C9" t="n">
-        <v>7.738192918486144e-05</v>
+        <v>0.007776883883078574</v>
       </c>
     </row>
     <row r="10">
@@ -547,7 +547,7 @@
         <v>242</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8291938537401489</v>
+        <v>0.4173156342182891</v>
       </c>
     </row>
     <row r="11">
@@ -560,7 +560,7 @@
         <v>615</v>
       </c>
       <c r="C11" t="n">
-        <v>0.8292038066572475</v>
+        <v>0.4183159023866989</v>
       </c>
     </row>
     <row r="12">
@@ -573,7 +573,7 @@
         <v>14167</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9951983178769601</v>
+        <v>0.5174309466344864</v>
       </c>
     </row>
     <row r="13">
@@ -586,7 +586,7 @@
         <v>1320</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9950600977413816</v>
+        <v>0.5035398230088496</v>
       </c>
     </row>
     <row r="14">
@@ -599,7 +599,7 @@
         <v>93</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8291898779099941</v>
+        <v>0.4169160632877447</v>
       </c>
     </row>
     <row r="15">
@@ -612,7 +612,7 @@
         <v>1079</v>
       </c>
       <c r="C15" t="n">
-        <v>2.879141434153983e-05</v>
+        <v>0.002893537141324752</v>
       </c>
     </row>
     <row r="16">
@@ -625,7 +625,7 @@
         <v>200</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9950302123066619</v>
+        <v>0.5005363368195227</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         <v>11420</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9952490163822881</v>
+        <v>0.5225261464199518</v>
       </c>
     </row>
     <row r="18">
@@ -651,7 +651,7 @@
         <v>711</v>
       </c>
       <c r="C18" t="n">
-        <v>0.8292063682659376</v>
+        <v>0.4185733440600697</v>
       </c>
     </row>
     <row r="19">
@@ -664,7 +664,7 @@
         <v>148</v>
       </c>
       <c r="C19" t="n">
-        <v>3.949146730813618e-06</v>
+        <v>0.0003968892464467686</v>
       </c>
     </row>
     <row r="20">
@@ -677,7 +677,7 @@
         <v>20000</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0005336684771369754</v>
+        <v>0.05363368195226603</v>
       </c>
     </row>
     <row r="21">
@@ -690,7 +690,7 @@
         <v>12000</v>
       </c>
       <c r="C21" t="n">
-        <v>0.0003202010862821853</v>
+        <v>0.03218020917135962</v>
       </c>
     </row>
     <row r="22">
@@ -703,7 +703,7 @@
         <v>5889.000000000001</v>
       </c>
       <c r="C22" t="n">
-        <v>0.995180439982976</v>
+        <v>0.5156342182890855</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         <v>4000</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0001067336954273951</v>
+        <v>0.01072673639045321</v>
       </c>
     </row>
     <row r="24">
@@ -729,7 +729,7 @@
         <v>4569</v>
       </c>
       <c r="C24" t="n">
-        <v>0.000121916563601942</v>
+        <v>0.01225261464199517</v>
       </c>
     </row>
     <row r="25">
@@ -742,7 +742,7 @@
         <v>3188</v>
       </c>
       <c r="C25" t="n">
-        <v>8.506675525563387e-05</v>
+        <v>0.008549208903191203</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         <v>4770</v>
       </c>
       <c r="C26" t="n">
-        <v>0.0001272799317971686</v>
+        <v>0.01279163314561545</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         <v>6500</v>
       </c>
       <c r="C27" t="n">
-        <v>0.000173442255069517</v>
+        <v>0.01743094663448646</v>
       </c>
     </row>
     <row r="28">
@@ -781,7 +781,7 @@
         <v>900</v>
       </c>
       <c r="C28" t="n">
-        <v>2.401508147116389e-05</v>
+        <v>0.002413515687851971</v>
       </c>
     </row>
     <row r="29">
@@ -794,7 +794,7 @@
         <v>752</v>
       </c>
       <c r="C29" t="n">
-        <v>0.9950248756218906</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="30">
@@ -807,7 +807,7 @@
         <v>8500</v>
       </c>
       <c r="C30" t="n">
-        <v>0.9952516847246737</v>
+        <v>0.5227943148297131</v>
       </c>
     </row>
     <row r="31">
@@ -820,7 +820,7 @@
         <v>6000</v>
       </c>
       <c r="C31" t="n">
-        <v>0.0001601005431410926</v>
+        <v>0.01609010458567981</v>
       </c>
     </row>
     <row r="32">
@@ -833,7 +833,7 @@
         <v>289</v>
       </c>
       <c r="C32" t="n">
-        <v>7.711509494629296e-06</v>
+        <v>0.0007750067042102441</v>
       </c>
     </row>
     <row r="33">
@@ -846,7 +846,7 @@
         <v>27000</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0007204524441349169</v>
+        <v>0.07240547063555913</v>
       </c>
     </row>
     <row r="34">
@@ -859,7 +859,7 @@
         <v>2900</v>
       </c>
       <c r="C34" t="n">
-        <v>7.738192918486144e-05</v>
+        <v>0.007776883883078574</v>
       </c>
     </row>
     <row r="35">
@@ -872,7 +872,7 @@
         <v>74580</v>
       </c>
       <c r="C35" t="n">
-        <v>0.9970149253731343</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="36">
@@ -885,7 +885,7 @@
         <v>7747</v>
       </c>
       <c r="C36" t="n">
-        <v>0.0002067164846190074</v>
+        <v>0.02077500670421024</v>
       </c>
     </row>
     <row r="37">
@@ -898,7 +898,7 @@
         <v>4239</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0001131110337291819</v>
+        <v>0.01136765888978278</v>
       </c>
     </row>
     <row r="38">
@@ -911,7 +911,7 @@
         <v>9200</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0002454874994830087</v>
+        <v>0.02467149369804237</v>
       </c>
     </row>
     <row r="39">
@@ -924,7 +924,7 @@
         <v>10000</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0002668342385684877</v>
+        <v>0.02681684097613301</v>
       </c>
     </row>
     <row r="40">
@@ -937,7 +937,7 @@
         <v>12000</v>
       </c>
       <c r="C40" t="n">
-        <v>0.0003202010862821853</v>
+        <v>0.03218020917135962</v>
       </c>
     </row>
     <row r="41">
@@ -950,7 +950,7 @@
         <v>3005</v>
       </c>
       <c r="C41" t="n">
-        <v>8.018368868983056e-05</v>
+        <v>0.00805846071332797</v>
       </c>
     </row>
     <row r="42">
@@ -963,7 +963,7 @@
         <v>5318</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0001419024480707218</v>
+        <v>0.01426119603110754</v>
       </c>
     </row>
     <row r="43">
@@ -976,7 +976,7 @@
         <v>6634</v>
       </c>
       <c r="C43" t="n">
-        <v>0.0001770178338663347</v>
+        <v>0.01779029230356664</v>
       </c>
     </row>
     <row r="44">
@@ -989,7 +989,7 @@
         <v>5866</v>
       </c>
       <c r="C44" t="n">
-        <v>0.0001565249643442749</v>
+        <v>0.01573075891659962</v>
       </c>
     </row>
     <row r="45">
@@ -1002,7 +1002,7 @@
         <v>290</v>
       </c>
       <c r="C45" t="n">
-        <v>0.8291951345444939</v>
+        <v>0.4174443550549746</v>
       </c>
     </row>
     <row r="46">
@@ -1015,7 +1015,7 @@
         <v>4000</v>
       </c>
       <c r="C46" t="n">
-        <v>0.0001067336954273951</v>
+        <v>0.01072673639045321</v>
       </c>
     </row>
     <row r="47">
@@ -1028,7 +1028,7 @@
         <v>14000</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0003735679339958828</v>
+        <v>0.03754357736658622</v>
       </c>
     </row>
     <row r="48">
@@ -1041,7 +1041,7 @@
         <v>6076</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0001621284833542131</v>
+        <v>0.01629391257709842</v>
       </c>
     </row>
     <row r="49">
@@ -1054,7 +1054,7 @@
         <v>5181</v>
       </c>
       <c r="C49" t="n">
-        <v>0.0001382468190023335</v>
+        <v>0.01389380530973451</v>
       </c>
     </row>
     <row r="50">
@@ -1067,7 +1067,7 @@
         <v>5113</v>
       </c>
       <c r="C50" t="n">
-        <v>0.8291873963515755</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
     <row r="51">
@@ -1080,7 +1080,7 @@
         <v>1000</v>
       </c>
       <c r="C51" t="n">
-        <v>0.9950515590457474</v>
+        <v>0.5026816840976133</v>
       </c>
     </row>
     <row r="52">
@@ -1093,7 +1093,7 @@
         <v>300</v>
       </c>
       <c r="C52" t="n">
-        <v>8.005027157054633e-06</v>
+        <v>0.0008045052292839904</v>
       </c>
     </row>
     <row r="53">
@@ -1106,7 +1106,7 @@
         <v>5703</v>
       </c>
       <c r="C53" t="n">
-        <v>0.0001521755662556085</v>
+        <v>0.01529364440868866</v>
       </c>
     </row>
     <row r="54">
@@ -1119,7 +1119,7 @@
         <v>1524</v>
       </c>
       <c r="C54" t="n">
-        <v>4.066553795783753e-05</v>
+        <v>0.004086886564762671</v>
       </c>
     </row>
     <row r="55">
@@ -1132,7 +1132,7 @@
         <v>2362</v>
       </c>
       <c r="C55" t="n">
-        <v>0.8292504225987253</v>
+        <v>0.4230008045052293</v>
       </c>
     </row>
     <row r="56">
@@ -1145,7 +1145,7 @@
         <v>421</v>
       </c>
       <c r="C56" t="n">
-        <v>1.123372144373333e-05</v>
+        <v>0.0011289890050952</v>
       </c>
     </row>
     <row r="57">
@@ -1158,7 +1158,7 @@
         <v>6492</v>
       </c>
       <c r="C57" t="n">
-        <v>0.0001732287876786622</v>
+        <v>0.01740949316170555</v>
       </c>
     </row>
     <row r="58">
@@ -1171,7 +1171,7 @@
         <v>2515</v>
       </c>
       <c r="C58" t="n">
-        <v>6.710881099997466e-05</v>
+        <v>0.006744435505497453</v>
       </c>
     </row>
     <row r="59">
@@ -1184,7 +1184,7 @@
         <v>3200</v>
       </c>
       <c r="C59" t="n">
-        <v>0.9951102625782325</v>
+        <v>0.5085813891123626</v>
       </c>
     </row>
     <row r="60">
@@ -1197,7 +1197,7 @@
         <v>1273</v>
       </c>
       <c r="C60" t="n">
-        <v>0.8292213643501453</v>
+        <v>0.4200804505229284</v>
       </c>
     </row>
     <row r="61">
@@ -1210,7 +1210,7 @@
         <v>4202</v>
       </c>
       <c r="C61" t="n">
-        <v>0.829299520098622</v>
+        <v>0.4279351032448378</v>
       </c>
     </row>
     <row r="62">
@@ -1223,7 +1223,7 @@
         <v>2618</v>
       </c>
       <c r="C62" t="n">
-        <v>0.8292572535552327</v>
+        <v>0.4236873156342183</v>
       </c>
     </row>
     <row r="63">
@@ -1236,7 +1236,7 @@
         <v>1379</v>
       </c>
       <c r="C63" t="n">
-        <v>3.679644149859446e-05</v>
+        <v>0.003698042370608742</v>
       </c>
     </row>
     <row r="64">
@@ -1249,7 +1249,7 @@
         <v>1295</v>
       </c>
       <c r="C64" t="n">
-        <v>0.8292219513854701</v>
+        <v>0.4201394475730759</v>
       </c>
     </row>
     <row r="65">
@@ -1262,7 +1262,7 @@
         <v>1386</v>
       </c>
       <c r="C65" t="n">
-        <v>0.8292243795770411</v>
+        <v>0.4203834808259587</v>
       </c>
     </row>
     <row r="66">
@@ -1275,7 +1275,7 @@
         <v>909</v>
       </c>
       <c r="C66" t="n">
-        <v>0.8292116515838613</v>
+        <v>0.4191043175113972</v>
       </c>
     </row>
     <row r="67">
@@ -1288,7 +1288,7 @@
         <v>1557</v>
       </c>
       <c r="C67" t="n">
-        <v>4.154609094511353e-05</v>
+        <v>0.00417538213998391</v>
       </c>
     </row>
     <row r="68">
@@ -1301,7 +1301,7 @@
         <v>2500</v>
       </c>
       <c r="C68" t="n">
-        <v>0.9950915841815327</v>
+        <v>0.5067042102440332</v>
       </c>
     </row>
     <row r="69">
@@ -1314,7 +1314,7 @@
         <v>2500</v>
       </c>
       <c r="C69" t="n">
-        <v>6.670855964212192e-05</v>
+        <v>0.006704210244033253</v>
       </c>
     </row>
     <row r="70">
@@ -1327,7 +1327,7 @@
         <v>12000</v>
       </c>
       <c r="C70" t="n">
-        <v>0.0003202010862821853</v>
+        <v>0.03218020917135962</v>
       </c>
     </row>
     <row r="71">
@@ -1340,7 +1340,7 @@
         <v>456</v>
       </c>
       <c r="C71" t="n">
-        <v>1.216764127872304e-05</v>
+        <v>0.001222847948511665</v>
       </c>
     </row>
     <row r="72">
@@ -1353,7 +1353,7 @@
         <v>4924</v>
       </c>
       <c r="C72" t="n">
-        <v>0.0001313891790711233</v>
+        <v>0.01320461249664789</v>
       </c>
     </row>
     <row r="73">
@@ -1366,7 +1366,7 @@
         <v>2136</v>
       </c>
       <c r="C73" t="n">
-        <v>5.699579335822898e-05</v>
+        <v>0.005728077232502012</v>
       </c>
     </row>
     <row r="74">
@@ -1379,7 +1379,7 @@
         <v>300</v>
       </c>
       <c r="C74" t="n">
-        <v>8.005027157054633e-06</v>
+        <v>0.0008045052292839904</v>
       </c>
     </row>
     <row r="75">
@@ -1392,7 +1392,7 @@
         <v>1034</v>
       </c>
       <c r="C75" t="n">
-        <v>0.8291873963515755</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
     <row r="76">
@@ -1405,7 +1405,7 @@
         <v>11</v>
       </c>
       <c r="C76" t="n">
-        <v>0.8291876898692379</v>
+        <v>0.4166961651917404</v>
       </c>
     </row>
     <row r="77">
@@ -1418,7 +1418,7 @@
         <v>1314</v>
       </c>
       <c r="C77" t="n">
-        <v>3.506201894789929e-05</v>
+        <v>0.003523732904263878</v>
       </c>
     </row>
     <row r="78">
@@ -1431,7 +1431,7 @@
         <v>609</v>
       </c>
       <c r="C78" t="n">
-        <v>1.62502051288209e-05</v>
+        <v>0.001633145615446501</v>
       </c>
     </row>
     <row r="79">
@@ -1444,7 +1444,7 @@
         <v>7000</v>
       </c>
       <c r="C79" t="n">
-        <v>0.0001867839669979414</v>
+        <v>0.01877178868329311</v>
       </c>
     </row>
     <row r="80">
@@ -1457,7 +1457,7 @@
         <v>2000</v>
       </c>
       <c r="C80" t="n">
-        <v>5.336684771369755e-05</v>
+        <v>0.005363368195226603</v>
       </c>
     </row>
     <row r="81">
@@ -1470,7 +1470,7 @@
         <v>17000</v>
       </c>
       <c r="C81" t="n">
-        <v>0.9953450767081727</v>
+        <v>0.5321802091713597</v>
       </c>
     </row>
     <row r="82">
@@ -1483,7 +1483,7 @@
         <v>951</v>
       </c>
       <c r="C82" t="n">
-        <v>0.8292127722876633</v>
+        <v>0.4192169482434969</v>
       </c>
     </row>
     <row r="83">
@@ -1496,7 +1496,7 @@
         <v>12</v>
       </c>
       <c r="C83" t="n">
-        <v>0.8291877165526618</v>
+        <v>0.416698846875838</v>
       </c>
     </row>
     <row r="84">
@@ -1509,7 +1509,7 @@
         <v>2778</v>
       </c>
       <c r="C84" t="n">
-        <v>0.8292080493216406</v>
+        <v>0.4187422901582194</v>
       </c>
     </row>
     <row r="85">
@@ -1522,7 +1522,7 @@
         <v>909</v>
       </c>
       <c r="C85" t="n">
-        <v>0.8292116515838613</v>
+        <v>0.4191043175113972</v>
       </c>
     </row>
     <row r="86">
@@ -1535,7 +1535,7 @@
         <v>536</v>
       </c>
       <c r="C86" t="n">
-        <v>0.8291873963515755</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
     <row r="87">
@@ -1548,7 +1548,7 @@
         <v>651</v>
       </c>
       <c r="C87" t="n">
-        <v>1.737090893080855e-05</v>
+        <v>0.001745776347546259</v>
       </c>
     </row>
     <row r="88">
@@ -1561,7 +1561,7 @@
         <v>6098</v>
       </c>
       <c r="C88" t="n">
-        <v>0.0001627155186790638</v>
+        <v>0.01635290962724591</v>
       </c>
     </row>
     <row r="89">
@@ -1574,7 +1574,7 @@
         <v>558</v>
       </c>
       <c r="C89" t="n">
-        <v>0.8292022857020875</v>
+        <v>0.4181630463931349</v>
       </c>
     </row>
     <row r="90">
@@ -1587,7 +1587,7 @@
         <v>5000</v>
       </c>
       <c r="C90" t="n">
-        <v>0.0001334171192842438</v>
+        <v>0.01340842048806651</v>
       </c>
     </row>
     <row r="91">
@@ -1600,7 +1600,7 @@
         <v>1586</v>
       </c>
       <c r="C91" t="n">
-        <v>4.231991023696216e-05</v>
+        <v>0.004253150978814696</v>
       </c>
     </row>
     <row r="92">
@@ -1613,7 +1613,7 @@
         <v>20</v>
       </c>
       <c r="C92" t="n">
-        <v>0.8291879300200526</v>
+        <v>0.416720300348619</v>
       </c>
     </row>
     <row r="93">
@@ -1626,7 +1626,7 @@
         <v>40</v>
       </c>
       <c r="C93" t="n">
-        <v>0.8291884636885297</v>
+        <v>0.4167739340305712</v>
       </c>
     </row>
     <row r="94">
@@ -1639,7 +1639,7 @@
         <v>102</v>
       </c>
       <c r="C94" t="n">
-        <v>0.8291900113271135</v>
+        <v>0.4169294717082328</v>
       </c>
     </row>
     <row r="95">
@@ -1652,7 +1652,7 @@
         <v>12000</v>
       </c>
       <c r="C95" t="n">
-        <v>0.0003202010862821853</v>
+        <v>0.03218020917135962</v>
       </c>
     </row>
     <row r="96">
@@ -1665,7 +1665,7 @@
         <v>300</v>
       </c>
       <c r="C96" t="n">
-        <v>8.005027157054633e-06</v>
+        <v>0.0008045052292839904</v>
       </c>
     </row>
     <row r="97">
@@ -1678,7 +1678,7 @@
         <v>17000</v>
       </c>
       <c r="C97" t="n">
-        <v>0.0004536182055664291</v>
+        <v>0.04558862965942612</v>
       </c>
     </row>
     <row r="98">
@@ -1691,7 +1691,7 @@
         <v>300</v>
       </c>
       <c r="C98" t="n">
-        <v>8.005027157054633e-06</v>
+        <v>0.0008045052292839904</v>
       </c>
     </row>
     <row r="99">
@@ -1704,7 +1704,7 @@
         <v>19000</v>
       </c>
       <c r="C99" t="n">
-        <v>0.0005069850532801267</v>
+        <v>0.05095199785465272</v>
       </c>
     </row>
     <row r="100">
@@ -1717,7 +1717,7 @@
         <v>4000</v>
       </c>
       <c r="C100" t="n">
-        <v>0.0001067336954273951</v>
+        <v>0.01072673639045321</v>
       </c>
     </row>
     <row r="101">
@@ -1730,7 +1730,7 @@
         <v>1003</v>
       </c>
       <c r="C101" t="n">
-        <v>0.8292141598257039</v>
+        <v>0.4193563958165728</v>
       </c>
     </row>
     <row r="102">
@@ -1743,7 +1743,7 @@
         <v>26</v>
       </c>
       <c r="C102" t="n">
-        <v>0.8291880901205957</v>
+        <v>0.4167363904532047</v>
       </c>
     </row>
     <row r="103">
@@ -1756,7 +1756,7 @@
         <v>456</v>
       </c>
       <c r="C103" t="n">
-        <v>0.8291995639928542</v>
+        <v>0.4178895146151784</v>
       </c>
     </row>
     <row r="104">
@@ -1769,7 +1769,7 @@
         <v>2500</v>
       </c>
       <c r="C104" t="n">
-        <v>0.8291873963515755</v>
+        <v>0.4166666666666667</v>
       </c>
     </row>
     <row r="105">
@@ -1782,7 +1782,7 @@
         <v>2500</v>
       </c>
       <c r="C105" t="n">
-        <v>6.670855964212192e-05</v>
+        <v>0.006704210244033253</v>
       </c>
     </row>
     <row r="106">
@@ -1795,7 +1795,7 @@
         <v>8000</v>
       </c>
       <c r="C106" t="n">
-        <v>0.0002134673908547902</v>
+        <v>0.02145347278090641</v>
       </c>
     </row>
     <row r="107">
@@ -1808,7 +1808,7 @@
         <v>579</v>
       </c>
       <c r="C107" t="n">
-        <v>1.544970241311544e-05</v>
+        <v>0.001552695092518101</v>
       </c>
     </row>
     <row r="108">
@@ -1821,7 +1821,7 @@
         <v>2847</v>
       </c>
       <c r="C108" t="n">
-        <v>7.596770772044846e-05</v>
+        <v>0.007634754625905069</v>
       </c>
     </row>
     <row r="109">
@@ -1834,7 +1834,7 @@
         <v>3274</v>
       </c>
       <c r="C109" t="n">
-        <v>8.736152970732288e-05</v>
+        <v>0.008779833735585949</v>
       </c>
     </row>
     <row r="110">
@@ -1847,7 +1847,7 @@
         <v>1113</v>
       </c>
       <c r="C110" t="n">
-        <v>0.8292170950023281</v>
+        <v>0.4196513810673103</v>
       </c>
     </row>
     <row r="111">
@@ -1860,7 +1860,7 @@
         <v>3325</v>
       </c>
       <c r="C111" t="n">
-        <v>0.8292227518881857</v>
+        <v>0.4202198980960043</v>
       </c>
     </row>
     <row r="112">
@@ -1873,7 +1873,7 @@
         <v>9000</v>
       </c>
       <c r="C112" t="n">
-        <v>0.0002401508147116389</v>
+        <v>0.02413515687851971</v>
       </c>
     </row>
     <row r="113">
@@ -1886,7 +1886,7 @@
         <v>3000</v>
       </c>
       <c r="C113" t="n">
-        <v>8.005027157054632e-05</v>
+        <v>0.008045052292839904</v>
       </c>
     </row>
     <row r="114">
@@ -1899,7 +1899,7 @@
         <v>1500</v>
       </c>
       <c r="C114" t="n">
-        <v>4.002513578527316e-05</v>
+        <v>0.004022526146419952</v>
       </c>
     </row>
     <row r="115">
@@ -1912,7 +1912,7 @@
         <v>30360</v>
       </c>
       <c r="C115" t="n">
-        <v>0.9958349843701845</v>
+        <v>0.5814159292035398</v>
       </c>
     </row>
     <row r="116">
@@ -1925,7 +1925,7 @@
         <v>25800</v>
       </c>
       <c r="C116" t="n">
-        <v>0.9957133079573973</v>
+        <v>0.5691874497184232</v>
       </c>
     </row>
     <row r="117">
@@ -1938,7 +1938,7 @@
         <v>29040</v>
       </c>
       <c r="C117" t="n">
-        <v>0.9957997622506934</v>
+        <v>0.5778761061946902</v>
       </c>
     </row>
     <row r="118">
@@ -1951,7 +1951,7 @@
         <v>300</v>
       </c>
       <c r="C118" t="n">
-        <v>0.9950328806490476</v>
+        <v>0.500804505229284</v>
       </c>
     </row>
     <row r="119">
@@ -1964,7 +1964,7 @@
         <v>3000</v>
       </c>
       <c r="C119" t="n">
-        <v>8.005027157054632e-05</v>
+        <v>0.008045052292839904</v>
       </c>
     </row>
     <row r="120">
@@ -1977,7 +1977,7 @@
         <v>26000</v>
       </c>
       <c r="C120" t="n">
-        <v>0.9957186446421686</v>
+        <v>0.5697237865379459</v>
       </c>
     </row>
     <row r="121">
@@ -1990,7 +1990,7 @@
         <v>5148</v>
       </c>
       <c r="C121" t="n">
-        <v>0.9951182676053896</v>
+        <v>0.5093858943416466</v>
       </c>
     </row>
   </sheetData>

</xml_diff>